<commit_message>
[DCM] Añadido taxonomia de Bloom a la matriz
</commit_message>
<xml_diff>
--- a/Diseño curricular de las matemáticas/Actividad 1/Matriz_competencias_DCM.xlsx
+++ b/Diseño curricular de las matemáticas/Actividad 1/Matriz_competencias_DCM.xlsx
@@ -452,13 +452,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
@@ -466,6 +466,7 @@
     <col width="6" customWidth="1" min="9" max="9"/>
     <col width="6" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -486,57 +487,63 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Nivel de Bloom</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Instrumentos de evaluación</t>
         </is>
       </c>
-      <c r="E1" s="1" t="n"/>
       <c r="F1" s="1" t="n"/>
       <c r="G1" s="1" t="n"/>
       <c r="H1" s="1" t="n"/>
       <c r="I1" s="1" t="n"/>
       <c r="J1" s="1" t="n"/>
       <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
     </row>
     <row r="2" ht="190" customHeight="1">
       <c r="A2" s="2" t="n"/>
       <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="n"/>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Examen escrito</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Cuestionario (GeoGebra Classroom)</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Fichas de construcción en GeoGebra</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Libro de GeoGebra (trabajo en equipo)</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Exposición oral</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Mapa conceptual</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Observación sistemática (registro y Kanban)</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Coevaluación y autoevaluación (rúbrica)</t>
         </is>
@@ -559,12 +566,12 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Representar vectores en GeoGebra y operar con ellos (suma, producto por un número y producto escalar), interpretando geométricamente el resultado de cada operación.</t>
+          <t>El alumno ha representado vectores en GeoGebra y ha calculado su suma, su producto por un número y su producto escalar, interpretando geométricamente cada resultado.</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>Aplicar</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -577,11 +584,16 @@
           <t>X</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n"/>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H3" s="5" t="n"/>
       <c r="I3" s="5" t="n"/>
       <c r="J3" s="5" t="n"/>
       <c r="K3" s="5" t="n"/>
+      <c r="L3" s="5" t="n"/>
     </row>
     <row r="4" ht="95" customHeight="1">
       <c r="A4" s="4" t="n"/>
@@ -592,25 +604,30 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Comprobar con GeoGebra los cálculos hechos a mano del módulo, el ángulo entre dos vectores y la proyección ortogonal, argumentando el origen de las discrepancias.</t>
+          <t>El alumno ha comprobado con GeoGebra el módulo, el ángulo entre dos vectores y la proyección ortogonal calculados a mano, justificando el origen de las discrepancias.</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n"/>
+          <t>Evaluar</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H4" s="5" t="n"/>
       <c r="I4" s="5" t="n"/>
       <c r="J4" s="5" t="n"/>
       <c r="K4" s="5" t="n"/>
+      <c r="L4" s="5" t="n"/>
     </row>
     <row r="5" ht="95" customHeight="1">
       <c r="A5" s="4" t="n"/>
@@ -621,12 +638,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Resolver problemas de perpendicularidad y de cálculo de ángulos mediante el producto escalar, conectando su expresión en coordenadas con su significado geométrico.</t>
+          <t>El alumno ha resuelto problemas de perpendicularidad y de cálculo de ángulos aplicando el producto escalar y relacionando su expresión en coordenadas con su significado geométrico.</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>Aplicar</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -634,12 +651,17 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F5" s="5" t="n"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
       <c r="I5" s="5" t="n"/>
       <c r="J5" s="5" t="n"/>
       <c r="K5" s="5" t="n"/>
+      <c r="L5" s="5" t="n"/>
     </row>
     <row r="6" ht="95" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -659,25 +681,30 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Emplear una circunferencia goniométrica dinámica en GeoGebra (con un deslizador para el ángulo) para investigar cómo varían el seno, el coseno y la tangente en los cuatro cuadrantes.</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n"/>
+          <t>El alumno ha examinado en una circunferencia goniométrica dinámica de GeoGebra (con un deslizador para el ángulo) cómo varían el seno, el coseno y la tangente en los cuatro cuadrantes.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Analizar</t>
+        </is>
+      </c>
       <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H6" s="5" t="n"/>
       <c r="I6" s="5" t="n"/>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="n"/>
+      <c r="J6" s="5" t="n"/>
+      <c r="K6" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="n"/>
     </row>
     <row r="7" ht="95" customHeight="1">
       <c r="A7" s="4" t="n"/>
@@ -688,25 +715,30 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Formular, de forma guiada, conjeturas sobre identidades trigonométricas (fundamental, ángulo doble, ángulo suma) a partir de la construcción y demostrarlas después por escrito.</t>
+          <t>El alumno ha formulado, de forma guiada, conjeturas sobre identidades trigonométricas (fundamental, ángulo doble, ángulo suma) a partir de la construcción y las ha demostrado por escrito.</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
+          <t>Crear</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H7" s="5" t="n"/>
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
+      <c r="L7" s="5" t="n"/>
     </row>
     <row r="8" ht="95" customHeight="1">
       <c r="A8" s="4" t="n"/>
@@ -717,12 +749,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Obtener todas las soluciones de ecuaciones trigonométricas sencillas, tanto en [0°, 360°) como su expresión general, describiendo el procedimiento seguido.</t>
+          <t>El alumno ha resuelto ecuaciones trigonométricas sencillas obteniendo todas sus soluciones, tanto en [0°, 360°) como en forma general, y ha descrito el procedimiento seguido.</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>Aplicar</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -730,12 +762,17 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F8" s="5" t="n"/>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="n"/>
       <c r="I8" s="5" t="n"/>
       <c r="J8" s="5" t="n"/>
       <c r="K8" s="5" t="n"/>
+      <c r="L8" s="5" t="n"/>
     </row>
     <row r="9" ht="95" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -753,25 +790,30 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Elegir entre el teorema del seno y el del coseno según los datos de cada triángulo, valorando qué estrategia resulta más eficiente.</t>
+          <t>El alumno ha justificado la elección entre el teorema del seno y el del coseno según los datos de cada triángulo, valorando la eficiencia de cada estrategia.</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
+          <t>Evaluar</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H9" s="5" t="n"/>
       <c r="I9" s="5" t="n"/>
       <c r="J9" s="5" t="n"/>
       <c r="K9" s="5" t="n"/>
+      <c r="L9" s="5" t="n"/>
     </row>
     <row r="10" ht="95" customHeight="1">
       <c r="A10" s="4" t="n"/>
@@ -782,25 +824,30 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Obtener todas las soluciones de un triángulo dado por dos lados y el ángulo opuesto a uno de ellos (dos, una o ninguna), describiendo el procedimiento utilizado.</t>
+          <t>El alumno ha discriminado si un triángulo dado por dos lados y el ángulo opuesto a uno de ellos tiene dos, una o ninguna solución y ha calculado todas las soluciones, describiendo el procedimiento.</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="n"/>
+          <t>Analizar</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H10" s="5" t="n"/>
       <c r="I10" s="5" t="n"/>
       <c r="J10" s="5" t="n"/>
       <c r="K10" s="5" t="n"/>
+      <c r="L10" s="5" t="n"/>
     </row>
     <row r="11" ht="95" customHeight="1">
       <c r="A11" s="4" t="n"/>
@@ -811,25 +858,30 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Verificar en GeoGebra, arrastrando los vértices, la validez de los triángulos obtenidos analíticamente y argumentar por qué un caso no tiene solución.</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+          <t>El alumno ha verificado en GeoGebra, arrastrando los vértices, la validez de los triángulos obtenidos analíticamente y ha argumentado por qué un caso no tiene solución.</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Evaluar</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="G11" s="5" t="n"/>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H11" s="5" t="n"/>
       <c r="I11" s="5" t="n"/>
       <c r="J11" s="5" t="n"/>
       <c r="K11" s="5" t="n"/>
+      <c r="L11" s="5" t="n"/>
     </row>
     <row r="12" ht="95" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
@@ -849,25 +901,30 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Relacionar el vector director y el vector normal con las distintas ecuaciones de la recta, integrando vectores, trigonometría y geometría analítica en una visión de conjunto.</t>
+          <t>El alumno ha relacionado el vector director y el vector normal con las distintas ecuaciones de la recta, organizando en un mapa conceptual las conexiones entre vectores, trigonometría y geometría analítica.</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="n"/>
+          <t>Analizar</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
       <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="n"/>
+      <c r="I12" s="5" t="n"/>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="K12" s="5" t="n"/>
+      <c r="L12" s="5" t="n"/>
     </row>
     <row r="13" ht="95" customHeight="1">
       <c r="A13" s="4" t="n"/>
@@ -878,12 +935,12 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Estudiar la posición relativa de dos rectas y calcular ángulos entre rectas y distancias de un punto a una recta, aplicando el producto escalar.</t>
+          <t>El alumno ha determinado la posición relativa de dos rectas y ha calculado ángulos entre rectas y distancias de un punto a una recta aplicando el producto escalar.</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>Aplicar</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -891,12 +948,17 @@
           <t>X</t>
         </is>
       </c>
-      <c r="F13" s="5" t="n"/>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="G13" s="5" t="n"/>
       <c r="H13" s="5" t="n"/>
       <c r="I13" s="5" t="n"/>
       <c r="J13" s="5" t="n"/>
       <c r="K13" s="5" t="n"/>
+      <c r="L13" s="5" t="n"/>
     </row>
     <row r="14" ht="95" customHeight="1">
       <c r="A14" s="4" t="n"/>
@@ -907,25 +969,30 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Seleccionar la ecuación de la recta (vectorial, paramétrica, continua, general o explícita) más útil para cada problema, justificando la elección.</t>
+          <t>El alumno ha seleccionado la ecuación de la recta (vectorial, paramétrica, continua, general o explícita) más útil para cada problema, justificando su elección.</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="n"/>
+          <t>Evaluar</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H14" s="5" t="n"/>
       <c r="I14" s="5" t="n"/>
       <c r="J14" s="5" t="n"/>
       <c r="K14" s="5" t="n"/>
+      <c r="L14" s="5" t="n"/>
     </row>
     <row r="15" ht="95" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -944,25 +1011,30 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Diseñar un método de medida y un modelo a escala en GeoGebra para calcular una altura o distancia inaccesible del centro, evaluando su eficiencia frente a otros métodos.</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="n"/>
+          <t>El alumno ha diseñado un método de medida y ha construido un modelo a escala en GeoGebra para calcular una altura o distancia inaccesible del centro, valorando su eficiencia frente a otros métodos.</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Crear</t>
+        </is>
+      </c>
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G15" s="5" t="n"/>
       <c r="H15" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="I15" s="5" t="n"/>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J15" s="5" t="n"/>
       <c r="K15" s="5" t="n"/>
+      <c r="L15" s="5" t="n"/>
     </row>
     <row r="16" ht="95" customHeight="1">
       <c r="A16" s="4" t="n"/>
@@ -973,25 +1045,30 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Seleccionar el resultado más razonable de entre las medidas repetidas, valorando el efecto que tiene un error de un grado en el resultado final.</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="n"/>
+          <t>El alumno ha valorado el efecto de un error de un grado en el resultado final y ha seleccionado, entre las medidas repetidas, el resultado más razonable.</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Evaluar</t>
+        </is>
+      </c>
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="G16" s="5" t="n"/>
       <c r="H16" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="I16" s="5" t="n"/>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J16" s="5" t="n"/>
       <c r="K16" s="5" t="n"/>
+      <c r="L16" s="5" t="n"/>
     </row>
     <row r="17" ht="95" customHeight="1">
       <c r="A17" s="4" t="n"/>
@@ -1002,21 +1079,26 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Organizar en un libro de GeoGebra la construcción, los cálculos y la explicación del método, eligiendo las representaciones más claras para el resto de la clase.</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="n"/>
+          <t>El alumno ha elaborado un libro de GeoGebra que integra la construcción, los cálculos y la explicación del método, eligiendo las representaciones más claras para compartirlo con la clase.</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Crear</t>
+        </is>
+      </c>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="H17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="I17" s="5" t="n"/>
       <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="K17" s="5" t="n"/>
+      <c r="L17" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -1031,21 +1113,26 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Exponer oralmente el método y los resultados con orden, usando la terminología y la notación matemáticas con rigor.</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="n"/>
+          <t>El alumno ha explicado oralmente el método y los resultados con orden, utilizando la terminología y la notación matemáticas con rigor.</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Comprender</t>
+        </is>
+      </c>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
       <c r="G18" s="5" t="n"/>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="I18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="J18" s="5" t="n"/>
-      <c r="K18" s="5" t="inlineStr">
+      <c r="K18" s="5" t="n"/>
+      <c r="L18" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -1068,21 +1155,26 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Aceptar las conjeturas fallidas y los errores de medida como punto de partida para revisar el razonamiento en la puesta en común.</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="n"/>
+          <t>El alumno ha analizado los errores de sus conjeturas y de sus medidas, y los ha utilizado como punto de partida para revisar su razonamiento en la puesta en común.</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Analizar</t>
+        </is>
+      </c>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
       <c r="G19" s="5" t="n"/>
       <c r="H19" s="5" t="n"/>
       <c r="I19" s="5" t="n"/>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J19" s="5" t="n"/>
       <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -1097,21 +1189,26 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Incorporar la crítica razonada recibida en la coevaluación para mejorar el libro de GeoGebra, sin abandonar ante las dificultades.</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="n"/>
+          <t>El alumno ha valorado la crítica razonada recibida en la coevaluación y la ha incorporado para mejorar el libro de GeoGebra, perseverando ante las dificultades.</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Evaluar</t>
+        </is>
+      </c>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
       <c r="G20" s="5" t="n"/>
       <c r="H20" s="5" t="n"/>
       <c r="I20" s="5" t="n"/>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J20" s="5" t="n"/>
       <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
@@ -1126,34 +1223,40 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Participar activamente en el equipo heterogéneo, asumiendo tareas en el tablero Kanban y escuchando los razonamientos de los compañeros.</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="n"/>
+          <t>El alumno ha colaborado activamente en el equipo heterogéneo, ha asumido tareas del tablero Kanban y ha tenido en cuenta los razonamientos de sus compañeros.</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Aplicar</t>
+        </is>
+      </c>
       <c r="E21" s="5" t="n"/>
       <c r="F21" s="5" t="n"/>
       <c r="G21" s="5" t="n"/>
       <c r="H21" s="5" t="n"/>
       <c r="I21" s="5" t="n"/>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
+      <c r="J21" s="5" t="n"/>
       <c r="K21" s="5" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A12:A14"/>
-    <mergeCell ref="D1:K1"/>
+    <mergeCell ref="E1:L1"/>
     <mergeCell ref="A3:A5"/>
     <mergeCell ref="A19:A21"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="B1:B2"/>
+    <mergeCell ref="D1:D2"/>
     <mergeCell ref="A15:A18"/>
     <mergeCell ref="A6:A8"/>
     <mergeCell ref="A9:A11"/>

</xml_diff>